<commit_message>
page permissions: the afternoon revision — purchasers near-manager, Locations owner only
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Page Permissions.xlsx
+++ b/docs/Page Permissions.xlsx
@@ -1454,9 +1454,7 @@
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
       <c r="E4" s="10"/>
-      <c r="F4" t="s" s="11">
-        <v>8</v>
-      </c>
+      <c r="F4" s="10"/>
       <c r="G4" t="s" s="11">
         <v>8</v>
       </c>
@@ -1762,7 +1760,7 @@
         <v>22</v>
       </c>
       <c r="E22" t="s" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F22" t="s" s="11">
         <v>8</v>
@@ -1802,7 +1800,7 @@
         <v>22</v>
       </c>
       <c r="E24" t="s" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F24" t="s" s="11">
         <v>8</v>
@@ -1821,7 +1819,7 @@
         <v>22</v>
       </c>
       <c r="E25" t="s" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F25" t="s" s="11">
         <v>8</v>
@@ -1842,7 +1840,7 @@
         <v>22</v>
       </c>
       <c r="E26" t="s" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F26" t="s" s="11">
         <v>8</v>
@@ -1990,7 +1988,7 @@
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" t="s" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F34" t="s" s="11">
         <v>8</v>
@@ -2043,7 +2041,7 @@
         <v>22</v>
       </c>
       <c r="E37" t="s" s="11">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="F37" t="s" s="11">
         <v>8</v>

</xml_diff>